<commit_message>
latest Code - Including the NDG/VUS flow
</commit_message>
<xml_diff>
--- a/UAA/src/src/test/resources/com/ugapp/data/testdata.xlsx
+++ b/UAA/src/src/test/resources/com/ugapp/data/testdata.xlsx
@@ -3,11 +3,11 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\divya\git\undergrad\UAA\src\src\test\resources\com\ugapp\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\divya\git\undergrad\UAA\src\src\test\resources\com\ugapp\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="9"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="test_suite" sheetId="1" r:id="rId1"/>
@@ -67,26 +67,6 @@
   </si>
   <si>
     <t>overAllAcademicsTest</t>
-  </si>
-  <si>
-    <t>Legal sex</t>
-  </si>
-  <si>
-    <t>X or another legal sex</t>
-  </si>
-  <si>
-    <t>Primary language spoken at home</t>
-  </si>
-  <si>
-    <t>Bavarian</t>
-  </si>
-  <si>
-    <t>Home address</t>
-  </si>
-  <si>
-    <t>Test Address line1 Test Address line2
-TestTestTestTestTestTestTestTest,Test State,Mayotte
-12345-678910</t>
   </si>
   <si>
     <t>email</t>
@@ -2397,25 +2377,25 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>67</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>1</v>
@@ -2423,25 +2403,25 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>3</v>
@@ -2449,25 +2429,25 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D3" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="G3" s="12" t="s">
         <v>72</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="F3" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>78</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>3</v>
@@ -2495,19 +2475,19 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>1</v>
@@ -2515,19 +2495,19 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>3</v>
@@ -2535,19 +2515,19 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>3</v>
@@ -2575,16 +2555,16 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -2592,16 +2572,16 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
@@ -2609,16 +2589,16 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -2642,16 +2622,16 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -2659,16 +2639,16 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C2" s="12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
@@ -2676,16 +2656,16 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -2693,16 +2673,16 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>3</v>
@@ -2710,16 +2690,16 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>3</v>
@@ -2727,16 +2707,16 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>3</v>
@@ -2744,16 +2724,16 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C7" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="D7" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>92</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>3</v>
@@ -2761,16 +2741,16 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>3</v>
@@ -2778,16 +2758,16 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>3</v>
@@ -2795,16 +2775,16 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>3</v>
@@ -2828,13 +2808,13 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
@@ -2842,13 +2822,13 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="11" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B2" s="11" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>3</v>
@@ -2856,13 +2836,13 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="12" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C3" s="13" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>3</v>
@@ -2870,13 +2850,13 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="12" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>3</v>
@@ -2885,10 +2865,10 @@
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="11"/>
       <c r="B5" s="12" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>3</v>
@@ -2897,10 +2877,10 @@
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="11"/>
       <c r="B6" s="12" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>3</v>
@@ -2928,16 +2908,16 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -2945,16 +2925,16 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
@@ -2962,16 +2942,16 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -3067,12 +3047,7 @@
       <c r="H7" s="3"/>
     </row>
     <row r="8" ht="14.25" customHeight="1">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>13</v>
-      </c>
+      <c r="B8" s="4"/>
       <c r="D8" s="3"/>
       <c r="E8" s="1"/>
       <c r="F8" s="3"/>
@@ -3081,12 +3056,7 @@
       <c r="L8" s="3"/>
     </row>
     <row r="9" ht="14.25" customHeight="1">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>15</v>
-      </c>
+      <c r="B9" s="4"/>
       <c r="D9" s="3"/>
       <c r="E9" s="1"/>
       <c r="F9" s="3"/>
@@ -3095,12 +3065,7 @@
       <c r="L9" s="3"/>
     </row>
     <row r="10" ht="137.25" customHeight="1">
-      <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>17</v>
-      </c>
+      <c r="B10" s="4"/>
       <c r="D10" s="3"/>
       <c r="E10" s="1"/>
       <c r="F10" s="3"/>
@@ -9278,10 +9243,10 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -9289,10 +9254,10 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="5" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>3</v>
@@ -9300,10 +9265,10 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="7" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>3</v>
@@ -9311,10 +9276,10 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="7" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
@@ -9342,16 +9307,16 @@
   <sheetData>
     <row r="1" ht="14.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -9359,16 +9324,16 @@
     </row>
     <row r="2" ht="14.25" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="D2" s="9" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
@@ -9376,16 +9341,16 @@
     </row>
     <row r="3" ht="14.25" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -9393,16 +9358,16 @@
     </row>
     <row r="4" ht="14.25" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>3</v>
@@ -9410,16 +9375,16 @@
     </row>
     <row r="5" ht="14.25" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="D5" s="9" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>3</v>
@@ -9427,16 +9392,16 @@
     </row>
     <row r="6" ht="14.25" customHeight="1">
       <c r="A6" s="9" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>3</v>
@@ -9460,16 +9425,16 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -9477,16 +9442,16 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D2" s="8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>3</v>
@@ -9494,16 +9459,16 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D3" s="8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>3</v>
@@ -9511,16 +9476,16 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="D4" s="8" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>3</v>
@@ -9528,16 +9493,16 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>3</v>
@@ -9563,10 +9528,10 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -9574,10 +9539,10 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>3</v>
@@ -9585,10 +9550,10 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>3</v>
@@ -9596,10 +9561,10 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
@@ -9607,10 +9572,10 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="9" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>3</v>
@@ -9618,10 +9583,10 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>3</v>
@@ -9629,10 +9594,10 @@
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>3</v>
@@ -9640,10 +9605,10 @@
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>3</v>
@@ -9651,10 +9616,10 @@
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>3</v>
@@ -9662,10 +9627,10 @@
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>3</v>
@@ -9673,10 +9638,10 @@
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>51</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>3</v>
@@ -9684,10 +9649,10 @@
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>3</v>
@@ -9695,10 +9660,10 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>3</v>
@@ -9706,10 +9671,10 @@
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="1" t="s">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>3</v>
@@ -9717,10 +9682,10 @@
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="1" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>3</v>
@@ -9746,10 +9711,10 @@
   <sheetData>
     <row r="1" ht="15" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -9757,10 +9722,10 @@
     </row>
     <row r="2" ht="15" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>3</v>
@@ -9768,10 +9733,10 @@
     </row>
     <row r="3" ht="15" customHeight="1">
       <c r="A3" s="6" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>3</v>
@@ -9779,10 +9744,10 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>3</v>
@@ -9790,10 +9755,10 @@
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>3</v>
@@ -9801,10 +9766,10 @@
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>3</v>

</xml_diff>